<commit_message>
docs: update requirements test and risk spreadsheets
</commit_message>
<xml_diff>
--- a/Phytium_PPE_System_SourceCode/功能需求表(表一).xlsx
+++ b/Phytium_PPE_System_SourceCode/功能需求表(表一).xlsx
@@ -53,7 +53,7 @@
     <t>USB摄像头实时拉流</t>
   </si>
   <si>
-    <t>通过 V4L2 驱动阻塞式拉取视频流，物理隔离在 Core 0 运行，保障 AI 算力。</t>
+    <t xml:space="preserve"> 基于 V4L2 持续读取视频帧，采集线程定向绑定 Core 0</t>
   </si>
   <si>
     <t>已实现 (帧率稳定)</t>
@@ -80,7 +80,7 @@
     <t>多线程无锁数据传输</t>
   </si>
   <si>
-    <t>采用 SPSC 无锁环形队列进行数据分发，基于 alignas(64) 消除伪共享。</t>
+    <t xml:space="preserve"> 原子无锁环形队列＋缓存行对齐，满载时主动丢弃新帧</t>
   </si>
   <si>
     <t>已实现 (纯用户态流转)</t>
@@ -95,10 +95,10 @@
     <t>PPE 八类目标检测</t>
   </si>
   <si>
-    <t>依托 NCNN 引擎与 INT8 量化模型，实现高保真 PPE 实时检测。</t>
-  </si>
-  <si>
-    <t>已实现 (mAP@0.5达80%)</t>
+    <t xml:space="preserve"> 采用 YOLOv8-NCNN INT8量化推理，检测安全帽、反光衣、手套和护目镜等目标</t>
+  </si>
+  <si>
+    <t>已实现 (mAP@0.5达76%)</t>
   </si>
   <si>
     <t>REQ-05</t>
@@ -107,7 +107,7 @@
     <t>复杂遮挡目标追踪</t>
   </si>
   <si>
-    <t>结合卡尔曼滤波与 ByteTrack 二次关联，维持极端遮挡工况下的 ID 稳定。</t>
+    <t xml:space="preserve"> ByteTrack低分框关联＋卡尔曼预测＋反向IoU标签挂载</t>
   </si>
   <si>
     <t>已实现 (抗遮挡性强)</t>
@@ -119,10 +119,10 @@
     <t>软硬联动模块</t>
   </si>
   <si>
-    <t>违规报警物理阻断</t>
-  </si>
-  <si>
-    <t>通过 OpenAMP RPMsg 协议驱动从核蜂鸣器，响应延迟达微秒级。</t>
+    <t>OpenAMP跨核告警</t>
+  </si>
+  <si>
+    <t>Linux主核通过RPMsg下发AI报警，从核完成CRC校验并控制蜂鸣器</t>
   </si>
   <si>
     <t>已实现 (异构联动成功)</t>
@@ -131,10 +131,10 @@
     <t>REQ-07</t>
   </si>
   <si>
-    <t>灾害环境硬中断与环境监测</t>
-  </si>
-  <si>
-    <t>从核实时监控火焰、有害气体（烟雾）及温湿度环境传感器，支持最高优先级硬件中断报警推送与高频数据采集。</t>
+    <t>裸机环境安全直通</t>
+  </si>
+  <si>
+    <t>火焰GPIO边沿中断直接触发本地报警，并采集MQ-2与AHT20数据</t>
   </si>
   <si>
     <t>已实现 (火焰、有害气体及温湿度传感器真机测试通过)</t>
@@ -146,10 +146,10 @@
     <t>UI交互渲染模块</t>
   </si>
   <si>
-    <t>零拷贝监控大屏</t>
-  </si>
-  <si>
-    <t>基于 Qt5 实现零拷贝图像渲染，动态叠加 OSD 报警框及置信度。</t>
+    <t>Qt5实时监控界面</t>
+  </si>
+  <si>
+    <t>低拷贝显示视频画面，动态叠加检测框、传感器与报警状态</t>
   </si>
   <si>
     <t>已实现 (渲染低延迟)</t>
@@ -158,10 +158,10 @@
     <t>REQ-09</t>
   </si>
   <si>
-    <t>硬件状态自视看板</t>
-  </si>
-  <si>
-    <t>解析 /proc/stat 动态展示 CPU 真实负载及核心热敏温度。</t>
+    <t>系统状态看板</t>
+  </si>
+  <si>
+    <t>读取CPU负载、内存占用、核心温度和RPMsg连接状态</t>
   </si>
   <si>
     <t>已实现 (数据动态刷新)</t>
@@ -173,10 +173,10 @@
     <t>本地存储模块</t>
   </si>
   <si>
-    <t>违规异步抓拍落盘</t>
-  </si>
-  <si>
-    <t>专职 I/O 线程后台执行 JPEG 编码与 CSV 记录，确保断电证据不丢失。</t>
+    <t>告警证据异步存储</t>
+  </si>
+  <si>
+    <t>独立I/O线程保存带OSD的告警截图，降低实时管线阻塞</t>
   </si>
   <si>
     <t>已实现 (IO 剥离成功)</t>
@@ -185,10 +185,10 @@
     <t>REQ-11</t>
   </si>
   <si>
-    <t>磁盘防洪自清洁机制</t>
-  </si>
-  <si>
-    <t>当磁盘占用超 85% 时自动启动循环覆盖，确保 system 长期无人值守运行。</t>
+    <t>磁盘水位保护</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 磁盘占用超过85%后周期清理旧证据，避免存储空间耗尽</t>
   </si>
   <si>
     <t>已实现 (自闭环运行)</t>
@@ -200,10 +200,10 @@
     <t>安全可靠性保障模块</t>
   </si>
   <si>
-    <t>主从核心跳通信</t>
-  </si>
-  <si>
-    <t>在 Linux 主核与 Bare-metal 从核间建立基于 OpenAMP RPMsg 的双向异步心跳通信，主核由独立 heartbeat_task 线程每 500ms 下发 DEVICE_CORE_CHECK 校验帧，从核实时监控主核业务存活状态以解决 SGI 邮箱中断丢失引起的僵死问题。</t>
+    <t>主从核心跳监测</t>
+  </si>
+  <si>
+    <t>500ms周期交换心跳，连续5s未收到主核消息后判定失联</t>
   </si>
   <si>
     <t>已实现 (Active Heartbeat心跳线程真机测试通过)</t>
@@ -212,13 +212,13 @@
     <t>REQ-13</t>
   </si>
   <si>
-    <t>看门狗(WDT)容错与自愈</t>
+    <t>FWDT硬件看门狗自愈</t>
   </si>
   <si>
     <t>在主核系统配置飞腾底层 FWDT 硬件看门狗，当主核宕机心跳超时（连续10次超时，共 5s）后，从核自动接管底层外设，进入 Fail-Safe 安全降级状态停止喂狗，在 1s WDT 超时后触发处理器硬件 cold reset 冷重启实现全面自愈。</t>
   </si>
   <si>
-    <t>已实现 (硬件看门狗超时10s冷重启真机测试通过)</t>
+    <t>已实现 (硬件看门狗超时1秒冷重启真机测试通过)</t>
   </si>
   <si>
     <t>REQ-14</t>
@@ -230,7 +230,7 @@
     <t>DeepSeek 研判与飞书联动推送</t>
   </si>
   <si>
-    <t>接入真实的 DeepSeek LLM API 生成智能化整改建议，规避表情符乱码并作聚合展示；同时通过后台独立子进程将违规警报及建议同步推送到绑定的飞书(Feishu)群聊中，且不阻塞主线程。</t>
+    <t>聚合违规事件，异步调用DeepSeek生成安全整改建议，并通过独立进程推送至飞书群</t>
   </si>
   <si>
     <t>已实现 (大模型研判及飞书异步推送测试通过)</t>

</xml_diff>